<commit_message>
create project schedule, risk management
</commit_message>
<xml_diff>
--- a/Project_ngan/01_Project_Management/BM01_NWS_P001_Project Open_v2.0.xlsx
+++ b/Project_ngan/01_Project_Management/BM01_NWS_P001_Project Open_v2.0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Documents\code-work\Newwave\BrSE_Training\AI_Training\Newwave_AI_Training\Project_ngan\01_Project_Management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D79FFD9A-47F7-4A02-9709-F61D8CA0E1B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27420358-B41E-4597-A11C-8A75917B3ACA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Thông tin chi tiết" sheetId="3" r:id="rId3"/>
     <sheet name="Master" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -1193,7 +1193,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="113">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1388,33 +1388,25 @@
     <xf numFmtId="0" fontId="22" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="12" fillId="6" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="18" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="15" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="14" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1425,26 +1417,8 @@
     <xf numFmtId="0" fontId="17" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="12" fillId="6" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="14" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1464,36 +1438,50 @@
     <xf numFmtId="0" fontId="16" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="18" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="15" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="11" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="5" borderId="11" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="11" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -1925,40 +1913,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="15.75" customHeight="1">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="85" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="80"/>
-      <c r="C1" s="80"/>
-      <c r="D1" s="80"/>
-      <c r="E1" s="80"/>
-      <c r="F1" s="80"/>
-      <c r="G1" s="80"/>
-      <c r="H1" s="80"/>
-      <c r="I1" s="80"/>
-      <c r="J1" s="80"/>
-      <c r="K1" s="80"/>
-      <c r="L1" s="80"/>
-      <c r="M1" s="80"/>
-      <c r="N1" s="80"/>
+      <c r="B1" s="85"/>
+      <c r="C1" s="85"/>
+      <c r="D1" s="85"/>
+      <c r="E1" s="85"/>
+      <c r="F1" s="85"/>
+      <c r="G1" s="85"/>
+      <c r="H1" s="85"/>
+      <c r="I1" s="85"/>
+      <c r="J1" s="85"/>
+      <c r="K1" s="85"/>
+      <c r="L1" s="85"/>
+      <c r="M1" s="85"/>
+      <c r="N1" s="85"/>
       <c r="O1" s="4"/>
       <c r="P1" s="4"/>
     </row>
     <row r="2" spans="1:16" ht="15.75" customHeight="1">
-      <c r="A2" s="80"/>
-      <c r="B2" s="80"/>
-      <c r="C2" s="80"/>
-      <c r="D2" s="80"/>
-      <c r="E2" s="80"/>
-      <c r="F2" s="80"/>
-      <c r="G2" s="80"/>
-      <c r="H2" s="80"/>
-      <c r="I2" s="80"/>
-      <c r="J2" s="80"/>
-      <c r="K2" s="80"/>
-      <c r="L2" s="80"/>
-      <c r="M2" s="80"/>
-      <c r="N2" s="80"/>
+      <c r="A2" s="85"/>
+      <c r="B2" s="85"/>
+      <c r="C2" s="85"/>
+      <c r="D2" s="85"/>
+      <c r="E2" s="85"/>
+      <c r="F2" s="85"/>
+      <c r="G2" s="85"/>
+      <c r="H2" s="85"/>
+      <c r="I2" s="85"/>
+      <c r="J2" s="85"/>
+      <c r="K2" s="85"/>
+      <c r="L2" s="85"/>
+      <c r="M2" s="85"/>
+      <c r="N2" s="85"/>
       <c r="O2" s="4"/>
       <c r="P2" s="4"/>
     </row>
@@ -2080,10 +2068,10 @@
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
-      <c r="D9" s="81"/>
-      <c r="E9" s="81"/>
-      <c r="F9" s="81"/>
-      <c r="G9" s="81"/>
+      <c r="D9" s="86"/>
+      <c r="E9" s="86"/>
+      <c r="F9" s="86"/>
+      <c r="G9" s="86"/>
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
@@ -2134,16 +2122,16 @@
       <c r="A12" s="5"/>
       <c r="B12" s="11"/>
       <c r="C12" s="15"/>
-      <c r="D12" s="82" t="s">
+      <c r="D12" s="87" t="s">
         <v>4</v>
       </c>
-      <c r="E12" s="82"/>
-      <c r="F12" s="82"/>
-      <c r="G12" s="82"/>
-      <c r="H12" s="82"/>
-      <c r="I12" s="82"/>
-      <c r="J12" s="82"/>
-      <c r="K12" s="82"/>
+      <c r="E12" s="87"/>
+      <c r="F12" s="87"/>
+      <c r="G12" s="87"/>
+      <c r="H12" s="87"/>
+      <c r="I12" s="87"/>
+      <c r="J12" s="87"/>
+      <c r="K12" s="87"/>
       <c r="L12" s="16"/>
       <c r="M12" s="6"/>
       <c r="N12" s="6"/>
@@ -2283,7 +2271,7 @@
       <c r="E19" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="F19" s="99" t="s">
+      <c r="F19" s="80" t="s">
         <v>110</v>
       </c>
       <c r="G19" s="28" t="s">
@@ -13774,35 +13762,35 @@
       <c r="A1" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="91" t="s">
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="89" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="91"/>
-      <c r="F1" s="91"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
       <c r="G1" s="32" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:7" s="33" customFormat="1" ht="17.25" customHeight="1">
       <c r="A2" s="31"/>
-      <c r="B2" s="90"/>
-      <c r="C2" s="90"/>
-      <c r="D2" s="91"/>
-      <c r="E2" s="91"/>
-      <c r="F2" s="91"/>
+      <c r="B2" s="88"/>
+      <c r="C2" s="88"/>
+      <c r="D2" s="89"/>
+      <c r="E2" s="89"/>
+      <c r="F2" s="89"/>
       <c r="G2" s="32" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="33" customFormat="1" ht="17.25" customHeight="1">
       <c r="A3" s="31"/>
-      <c r="B3" s="90"/>
-      <c r="C3" s="90"/>
-      <c r="D3" s="91"/>
-      <c r="E3" s="91"/>
-      <c r="F3" s="91"/>
+      <c r="B3" s="88"/>
+      <c r="C3" s="88"/>
+      <c r="D3" s="89"/>
+      <c r="E3" s="89"/>
+      <c r="F3" s="89"/>
       <c r="G3" s="32" t="s">
         <v>19</v>
       </c>
@@ -13834,22 +13822,22 @@
       <c r="B7" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="100" t="s">
+      <c r="C7" s="92" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="101"/>
-      <c r="E7" s="102"/>
+      <c r="D7" s="93"/>
+      <c r="E7" s="94"/>
     </row>
     <row r="8" spans="1:7" s="36" customFormat="1" ht="15.6">
       <c r="A8" s="34"/>
       <c r="B8" s="2">
         <v>1</v>
       </c>
-      <c r="C8" s="103" t="s">
+      <c r="C8" s="95" t="s">
         <v>111</v>
       </c>
-      <c r="D8" s="104"/>
-      <c r="E8" s="105"/>
+      <c r="D8" s="96"/>
+      <c r="E8" s="97"/>
       <c r="F8" s="35"/>
       <c r="G8" s="35"/>
     </row>
@@ -13881,14 +13869,14 @@
       <c r="C11" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="92" t="s">
+      <c r="D11" s="90" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="92"/>
-      <c r="F11" s="86" t="s">
+      <c r="E11" s="90"/>
+      <c r="F11" s="91" t="s">
         <v>26</v>
       </c>
-      <c r="G11" s="86"/>
+      <c r="G11" s="91"/>
     </row>
     <row r="12" spans="1:7" s="36" customFormat="1" ht="15.6">
       <c r="A12" s="34"/>
@@ -13898,14 +13886,14 @@
       <c r="C12" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="89" t="s">
+      <c r="D12" s="98" t="s">
         <v>107</v>
       </c>
-      <c r="E12" s="89"/>
-      <c r="F12" s="88" t="s">
+      <c r="E12" s="98"/>
+      <c r="F12" s="99" t="s">
         <v>112</v>
       </c>
-      <c r="G12" s="88"/>
+      <c r="G12" s="99"/>
     </row>
     <row r="13" spans="1:7" s="36" customFormat="1" ht="15.6">
       <c r="A13" s="34"/>
@@ -13919,10 +13907,10 @@
     </row>
     <row r="15" spans="1:7" s="36" customFormat="1" ht="15" customHeight="1">
       <c r="A15" s="34"/>
-      <c r="B15" s="85" t="s">
+      <c r="B15" s="100" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="85"/>
+      <c r="C15" s="100"/>
       <c r="D15" s="41" t="s">
         <v>30</v>
       </c>
@@ -13938,29 +13926,29 @@
     </row>
     <row r="16" spans="1:7" s="36" customFormat="1" ht="15" customHeight="1">
       <c r="A16" s="34"/>
-      <c r="B16" s="85" t="s">
+      <c r="B16" s="100" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="85"/>
+      <c r="C16" s="100"/>
       <c r="D16" s="41" t="s">
         <v>34</v>
       </c>
-      <c r="E16" s="106">
+      <c r="E16" s="81">
         <v>42200</v>
       </c>
       <c r="F16" s="43" t="s">
         <v>35</v>
       </c>
-      <c r="G16" s="106">
+      <c r="G16" s="81">
         <v>42221</v>
       </c>
     </row>
     <row r="17" spans="1:33" s="36" customFormat="1" ht="15" customHeight="1">
       <c r="A17" s="34"/>
-      <c r="B17" s="85" t="s">
+      <c r="B17" s="100" t="s">
         <v>36</v>
       </c>
-      <c r="C17" s="85"/>
+      <c r="C17" s="100"/>
       <c r="D17" s="41" t="s">
         <v>37</v>
       </c>
@@ -13988,10 +13976,10 @@
       <c r="E20" s="46" t="s">
         <v>41</v>
       </c>
-      <c r="F20" s="86"/>
-      <c r="G20" s="86"/>
-    </row>
-    <row r="21" spans="1:33" s="34" customFormat="1" ht="15.6">
+      <c r="F20" s="91"/>
+      <c r="G20" s="91"/>
+    </row>
+    <row r="21" spans="1:33" s="34" customFormat="1" ht="31.2">
       <c r="B21" s="47">
         <v>1</v>
       </c>
@@ -14004,8 +13992,8 @@
       <c r="E21" s="48" t="s">
         <v>117</v>
       </c>
-      <c r="F21" s="87"/>
-      <c r="G21" s="87"/>
+      <c r="F21" s="101"/>
+      <c r="G21" s="101"/>
     </row>
     <row r="22" spans="1:33" s="49" customFormat="1" ht="15.6">
       <c r="A22" s="34"/>
@@ -14019,8 +14007,8 @@
         <v>119</v>
       </c>
       <c r="E22" s="48"/>
-      <c r="F22" s="87"/>
-      <c r="G22" s="87"/>
+      <c r="F22" s="101"/>
+      <c r="G22" s="101"/>
       <c r="H22" s="34"/>
       <c r="I22" s="34"/>
       <c r="J22" s="34"/>
@@ -14127,10 +14115,10 @@
       <c r="C25" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="D25" s="83" t="s">
+      <c r="D25" s="102" t="s">
         <v>24</v>
       </c>
-      <c r="E25" s="83"/>
+      <c r="E25" s="102"/>
     </row>
     <row r="26" spans="1:33" s="34" customFormat="1" ht="15.6">
       <c r="B26" s="47">
@@ -14139,10 +14127,10 @@
       <c r="C26" s="50" t="s">
         <v>43</v>
       </c>
-      <c r="D26" s="84" t="s">
+      <c r="D26" s="103" t="s">
         <v>44</v>
       </c>
-      <c r="E26" s="84"/>
+      <c r="E26" s="103"/>
     </row>
     <row r="27" spans="1:33" s="34" customFormat="1" ht="15.6">
       <c r="B27" s="47">
@@ -14151,18 +14139,18 @@
       <c r="C27" s="50" t="s">
         <v>45</v>
       </c>
-      <c r="D27" s="84" t="s">
+      <c r="D27" s="103" t="s">
         <v>46</v>
       </c>
-      <c r="E27" s="84"/>
+      <c r="E27" s="103"/>
     </row>
     <row r="28" spans="1:33" s="34" customFormat="1" ht="15.6">
       <c r="B28" s="47">
         <v>3</v>
       </c>
       <c r="C28" s="50"/>
-      <c r="D28" s="84"/>
-      <c r="E28" s="84"/>
+      <c r="D28" s="103"/>
+      <c r="E28" s="103"/>
     </row>
     <row r="29" spans="1:33" s="34" customFormat="1" ht="15.6">
       <c r="B29" s="47">
@@ -14171,8 +14159,8 @@
       <c r="C29" s="51" t="s">
         <v>47</v>
       </c>
-      <c r="D29" s="84"/>
-      <c r="E29" s="84"/>
+      <c r="D29" s="103"/>
+      <c r="E29" s="103"/>
     </row>
     <row r="30" spans="1:33" s="49" customFormat="1" ht="15.6">
       <c r="A30" s="34"/>
@@ -14289,25 +14277,25 @@
     <row r="58" s="49" customFormat="1" ht="15.6"/>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
     <mergeCell ref="B1:C3"/>
     <mergeCell ref="D1:F3"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="F11:G11"/>
     <mergeCell ref="C7:E7"/>
     <mergeCell ref="C8:E8"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="D29:E29"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E15" xr:uid="{00000000-0002-0000-0100-000000000000}">
@@ -14346,13 +14334,13 @@
       <c r="A1" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="91" t="s">
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="89" t="s">
         <v>48</v>
       </c>
-      <c r="E1" s="91"/>
-      <c r="F1" s="91"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
       <c r="G1" s="32" t="str">
         <f>'Thông tin cơ bản'!G1</f>
         <v>Mã số: BM01-QT-OP-01</v>
@@ -14360,11 +14348,11 @@
     </row>
     <row r="2" spans="1:13" s="33" customFormat="1" ht="17.25" customHeight="1">
       <c r="A2" s="31"/>
-      <c r="B2" s="90"/>
-      <c r="C2" s="90"/>
-      <c r="D2" s="91"/>
-      <c r="E2" s="91"/>
-      <c r="F2" s="91"/>
+      <c r="B2" s="88"/>
+      <c r="C2" s="88"/>
+      <c r="D2" s="89"/>
+      <c r="E2" s="89"/>
+      <c r="F2" s="89"/>
       <c r="G2" s="32" t="str">
         <f>'Thông tin cơ bản'!G2</f>
         <v>Ngày hiệu lực: 10/09/2025</v>
@@ -14372,11 +14360,11 @@
     </row>
     <row r="3" spans="1:13" s="33" customFormat="1" ht="17.25" customHeight="1">
       <c r="A3" s="31"/>
-      <c r="B3" s="90"/>
-      <c r="C3" s="90"/>
-      <c r="D3" s="91"/>
-      <c r="E3" s="91"/>
-      <c r="F3" s="91"/>
+      <c r="B3" s="88"/>
+      <c r="C3" s="88"/>
+      <c r="D3" s="89"/>
+      <c r="E3" s="89"/>
+      <c r="F3" s="89"/>
       <c r="G3" s="32" t="str">
         <f>'Thông tin cơ bản'!G3</f>
         <v>Lần ban hành: 02</v>
@@ -14393,33 +14381,33 @@
     </row>
     <row r="7" spans="1:13" s="36" customFormat="1" ht="146.4" customHeight="1">
       <c r="A7" s="34"/>
-      <c r="B7" s="97" t="s">
+      <c r="B7" s="104" t="s">
         <v>50</v>
       </c>
-      <c r="C7" s="97"/>
+      <c r="C7" s="104"/>
       <c r="D7" s="53" t="s">
         <v>51</v>
       </c>
-      <c r="E7" s="98" t="s">
+      <c r="E7" s="105" t="s">
         <v>164</v>
       </c>
-      <c r="F7" s="98"/>
-      <c r="G7" s="98"/>
+      <c r="F7" s="105"/>
+      <c r="G7" s="105"/>
       <c r="H7" s="34"/>
       <c r="I7" s="34"/>
     </row>
     <row r="8" spans="1:13" s="36" customFormat="1" ht="171.75" customHeight="1">
       <c r="A8" s="34"/>
-      <c r="B8" s="97"/>
-      <c r="C8" s="97"/>
+      <c r="B8" s="104"/>
+      <c r="C8" s="104"/>
       <c r="D8" s="53" t="s">
         <v>52</v>
       </c>
-      <c r="E8" s="98" t="s">
+      <c r="E8" s="105" t="s">
         <v>165</v>
       </c>
-      <c r="F8" s="98"/>
-      <c r="G8" s="98"/>
+      <c r="F8" s="105"/>
+      <c r="G8" s="105"/>
       <c r="H8" s="34"/>
       <c r="I8" s="34"/>
     </row>
@@ -14632,101 +14620,101 @@
       <c r="C28" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="D28" s="83" t="s">
+      <c r="D28" s="102" t="s">
         <v>24</v>
       </c>
-      <c r="E28" s="83"/>
+      <c r="E28" s="102"/>
       <c r="H28" s="52"/>
     </row>
     <row r="29" spans="2:8" s="34" customFormat="1" ht="15.6">
       <c r="B29" s="47">
         <v>1</v>
       </c>
-      <c r="C29" s="107" t="s">
+      <c r="C29" s="82" t="s">
         <v>120</v>
       </c>
-      <c r="D29" s="108" t="s">
+      <c r="D29" s="106" t="s">
         <v>121</v>
       </c>
-      <c r="E29" s="108"/>
+      <c r="E29" s="106"/>
       <c r="H29" s="52"/>
     </row>
     <row r="30" spans="2:8" s="34" customFormat="1" ht="15.6">
       <c r="B30" s="47">
         <v>2</v>
       </c>
-      <c r="C30" s="107" t="s">
+      <c r="C30" s="82" t="s">
         <v>122</v>
       </c>
-      <c r="D30" s="108" t="s">
+      <c r="D30" s="106" t="s">
         <v>123</v>
       </c>
-      <c r="E30" s="108"/>
+      <c r="E30" s="106"/>
       <c r="H30" s="52"/>
     </row>
     <row r="31" spans="2:8" s="34" customFormat="1" ht="15.6">
       <c r="B31" s="47">
         <v>3</v>
       </c>
-      <c r="C31" s="107" t="s">
+      <c r="C31" s="82" t="s">
         <v>124</v>
       </c>
-      <c r="D31" s="108" t="s">
+      <c r="D31" s="106" t="s">
         <v>125</v>
       </c>
-      <c r="E31" s="108"/>
+      <c r="E31" s="106"/>
       <c r="H31" s="52"/>
     </row>
     <row r="32" spans="2:8" s="34" customFormat="1" ht="15.6">
       <c r="B32" s="47">
         <v>4</v>
       </c>
-      <c r="C32" s="107" t="s">
+      <c r="C32" s="82" t="s">
         <v>126</v>
       </c>
-      <c r="D32" s="108" t="s">
+      <c r="D32" s="106" t="s">
         <v>127</v>
       </c>
-      <c r="E32" s="108"/>
+      <c r="E32" s="106"/>
       <c r="H32" s="52"/>
     </row>
     <row r="33" spans="2:8" s="34" customFormat="1" ht="15.6">
       <c r="B33" s="47">
         <v>5</v>
       </c>
-      <c r="C33" s="107" t="s">
+      <c r="C33" s="82" t="s">
         <v>128</v>
       </c>
-      <c r="D33" s="84" t="s">
+      <c r="D33" s="103" t="s">
         <v>129</v>
       </c>
-      <c r="E33" s="84"/>
+      <c r="E33" s="103"/>
       <c r="H33" s="52"/>
     </row>
     <row r="34" spans="2:8" s="34" customFormat="1" ht="15.6">
       <c r="B34" s="47">
         <v>6</v>
       </c>
-      <c r="C34" s="107" t="s">
+      <c r="C34" s="82" t="s">
         <v>130</v>
       </c>
-      <c r="D34" s="84" t="s">
+      <c r="D34" s="103" t="s">
         <v>131</v>
       </c>
-      <c r="E34" s="84"/>
+      <c r="E34" s="103"/>
       <c r="H34" s="52"/>
     </row>
     <row r="35" spans="2:8" s="34" customFormat="1" ht="15.6">
       <c r="B35" s="47">
         <v>7</v>
       </c>
-      <c r="C35" s="107" t="s">
+      <c r="C35" s="82" t="s">
         <v>132</v>
       </c>
-      <c r="D35" s="84" t="s">
+      <c r="D35" s="103" t="s">
         <v>133</v>
       </c>
-      <c r="E35" s="84"/>
+      <c r="E35" s="103"/>
       <c r="H35" s="52"/>
     </row>
     <row r="36" spans="2:8" s="34" customFormat="1" ht="15.6">
@@ -14734,8 +14722,8 @@
         <v>8</v>
       </c>
       <c r="C36" s="51"/>
-      <c r="D36" s="84"/>
-      <c r="E36" s="84"/>
+      <c r="D36" s="103"/>
+      <c r="E36" s="103"/>
       <c r="H36" s="52"/>
     </row>
     <row r="37" spans="2:8" s="34" customFormat="1" ht="15.6">
@@ -14754,10 +14742,10 @@
       <c r="C39" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="D39" s="83" t="s">
+      <c r="D39" s="102" t="s">
         <v>74</v>
       </c>
-      <c r="E39" s="83"/>
+      <c r="E39" s="102"/>
       <c r="F39" s="55" t="s">
         <v>54</v>
       </c>
@@ -14770,10 +14758,10 @@
       <c r="C40" s="54" t="s">
         <v>134</v>
       </c>
-      <c r="D40" s="110" t="s">
+      <c r="D40" s="107" t="s">
         <v>135</v>
       </c>
-      <c r="E40" s="98"/>
+      <c r="E40" s="105"/>
       <c r="F40" s="54" t="s">
         <v>61</v>
       </c>
@@ -14786,10 +14774,10 @@
       <c r="C41" s="54" t="s">
         <v>75</v>
       </c>
-      <c r="D41" s="109" t="s">
+      <c r="D41" s="108" t="s">
         <v>117</v>
       </c>
-      <c r="E41" s="95"/>
+      <c r="E41" s="109"/>
       <c r="F41" s="54" t="s">
         <v>63</v>
       </c>
@@ -14816,367 +14804,367 @@
       <c r="C44" s="46" t="s">
         <v>77</v>
       </c>
-      <c r="D44" s="96" t="s">
+      <c r="D44" s="110" t="s">
         <v>78</v>
       </c>
-      <c r="E44" s="96"/>
+      <c r="E44" s="110"/>
       <c r="F44" s="46" t="s">
         <v>54</v>
       </c>
       <c r="H44" s="52"/>
     </row>
     <row r="45" spans="2:8" s="34" customFormat="1" ht="15.6">
-      <c r="B45" s="115">
+      <c r="B45" s="83">
         <v>1</v>
       </c>
-      <c r="C45" s="116" t="s">
+      <c r="C45" s="84" t="s">
         <v>136</v>
       </c>
-      <c r="D45" s="84"/>
-      <c r="E45" s="84"/>
-      <c r="F45" s="116" t="s">
+      <c r="D45" s="103"/>
+      <c r="E45" s="103"/>
+      <c r="F45" s="84" t="s">
         <v>136</v>
       </c>
       <c r="H45" s="52"/>
     </row>
     <row r="46" spans="2:8" s="34" customFormat="1" ht="15.6">
-      <c r="B46" s="115">
+      <c r="B46" s="83">
         <v>2</v>
       </c>
-      <c r="C46" s="116" t="s">
+      <c r="C46" s="84" t="s">
         <v>163</v>
       </c>
-      <c r="D46" s="84"/>
-      <c r="E46" s="84"/>
-      <c r="F46" s="116" t="s">
+      <c r="D46" s="103"/>
+      <c r="E46" s="103"/>
+      <c r="F46" s="84" t="s">
         <v>136</v>
       </c>
       <c r="H46" s="52"/>
     </row>
     <row r="47" spans="2:8" s="34" customFormat="1" ht="15.6">
-      <c r="B47" s="115">
+      <c r="B47" s="83">
         <v>3</v>
       </c>
-      <c r="C47" s="116" t="s">
+      <c r="C47" s="84" t="s">
         <v>137</v>
       </c>
-      <c r="D47" s="84"/>
-      <c r="E47" s="84"/>
-      <c r="F47" s="116" t="s">
+      <c r="D47" s="103"/>
+      <c r="E47" s="103"/>
+      <c r="F47" s="84" t="s">
         <v>136</v>
       </c>
       <c r="H47" s="52"/>
     </row>
     <row r="48" spans="2:8" s="34" customFormat="1" ht="15.6">
-      <c r="B48" s="115">
+      <c r="B48" s="83">
         <v>4</v>
       </c>
-      <c r="C48" s="116" t="s">
+      <c r="C48" s="84" t="s">
         <v>138</v>
       </c>
-      <c r="D48" s="84"/>
-      <c r="E48" s="84"/>
-      <c r="F48" s="116" t="s">
+      <c r="D48" s="103"/>
+      <c r="E48" s="103"/>
+      <c r="F48" s="84" t="s">
         <v>136</v>
       </c>
       <c r="H48" s="52"/>
     </row>
     <row r="49" spans="2:8" s="34" customFormat="1" ht="15.6">
-      <c r="B49" s="115">
+      <c r="B49" s="83">
         <v>5</v>
       </c>
-      <c r="C49" s="116" t="s">
+      <c r="C49" s="84" t="s">
         <v>139</v>
       </c>
-      <c r="D49" s="84"/>
-      <c r="E49" s="84"/>
-      <c r="F49" s="116" t="s">
+      <c r="D49" s="103"/>
+      <c r="E49" s="103"/>
+      <c r="F49" s="84" t="s">
         <v>136</v>
       </c>
       <c r="H49" s="52"/>
     </row>
     <row r="50" spans="2:8" s="34" customFormat="1" ht="15.6">
-      <c r="B50" s="115">
+      <c r="B50" s="83">
         <v>6</v>
       </c>
-      <c r="C50" s="116" t="s">
+      <c r="C50" s="84" t="s">
         <v>140</v>
       </c>
-      <c r="D50" s="84"/>
-      <c r="E50" s="84"/>
+      <c r="D50" s="103"/>
+      <c r="E50" s="103"/>
       <c r="F50" s="54"/>
       <c r="H50" s="52"/>
     </row>
     <row r="51" spans="2:8" s="34" customFormat="1" ht="15.6">
-      <c r="B51" s="115">
+      <c r="B51" s="83">
         <v>7</v>
       </c>
-      <c r="C51" s="116" t="s">
+      <c r="C51" s="84" t="s">
         <v>141</v>
       </c>
-      <c r="D51" s="84"/>
-      <c r="E51" s="84"/>
+      <c r="D51" s="103"/>
+      <c r="E51" s="103"/>
       <c r="F51" s="54"/>
       <c r="H51" s="52"/>
     </row>
     <row r="52" spans="2:8" s="34" customFormat="1" ht="15.6">
-      <c r="B52" s="115">
+      <c r="B52" s="83">
         <v>8</v>
       </c>
-      <c r="C52" s="116" t="s">
+      <c r="C52" s="84" t="s">
         <v>142</v>
       </c>
-      <c r="D52" s="84"/>
-      <c r="E52" s="84"/>
+      <c r="D52" s="103"/>
+      <c r="E52" s="103"/>
       <c r="F52" s="54"/>
       <c r="H52" s="52"/>
     </row>
     <row r="53" spans="2:8" s="34" customFormat="1" ht="15.6">
-      <c r="B53" s="115">
+      <c r="B53" s="83">
         <v>9</v>
       </c>
-      <c r="C53" s="116" t="s">
+      <c r="C53" s="84" t="s">
         <v>143</v>
       </c>
-      <c r="D53" s="84"/>
-      <c r="E53" s="84"/>
+      <c r="D53" s="103"/>
+      <c r="E53" s="103"/>
       <c r="F53" s="54"/>
       <c r="H53" s="52"/>
     </row>
     <row r="54" spans="2:8" s="34" customFormat="1" ht="15.6">
-      <c r="B54" s="115">
+      <c r="B54" s="83">
         <v>10</v>
       </c>
-      <c r="C54" s="116" t="s">
+      <c r="C54" s="84" t="s">
         <v>144</v>
       </c>
-      <c r="D54" s="84"/>
-      <c r="E54" s="84"/>
+      <c r="D54" s="103"/>
+      <c r="E54" s="103"/>
       <c r="F54" s="54"/>
       <c r="H54" s="52"/>
     </row>
     <row r="55" spans="2:8" s="34" customFormat="1" ht="15.6">
-      <c r="B55" s="115">
+      <c r="B55" s="83">
         <v>11</v>
       </c>
-      <c r="C55" s="116" t="s">
+      <c r="C55" s="84" t="s">
         <v>145</v>
       </c>
-      <c r="D55" s="84"/>
-      <c r="E55" s="84"/>
+      <c r="D55" s="103"/>
+      <c r="E55" s="103"/>
       <c r="F55" s="54"/>
       <c r="H55" s="52"/>
     </row>
     <row r="56" spans="2:8" s="34" customFormat="1" ht="15.6">
-      <c r="B56" s="115">
+      <c r="B56" s="83">
         <v>12</v>
       </c>
-      <c r="C56" s="116" t="s">
+      <c r="C56" s="84" t="s">
         <v>146</v>
       </c>
-      <c r="D56" s="84"/>
-      <c r="E56" s="84"/>
+      <c r="D56" s="103"/>
+      <c r="E56" s="103"/>
       <c r="F56" s="54"/>
       <c r="H56" s="52"/>
     </row>
     <row r="57" spans="2:8" s="34" customFormat="1" ht="15.6">
-      <c r="B57" s="115">
+      <c r="B57" s="83">
         <v>13</v>
       </c>
-      <c r="C57" s="116" t="s">
+      <c r="C57" s="84" t="s">
         <v>147</v>
       </c>
-      <c r="D57" s="84"/>
-      <c r="E57" s="84"/>
+      <c r="D57" s="103"/>
+      <c r="E57" s="103"/>
       <c r="F57" s="54"/>
       <c r="H57" s="52"/>
     </row>
     <row r="58" spans="2:8" s="34" customFormat="1" ht="15.6">
-      <c r="B58" s="115">
+      <c r="B58" s="83">
         <v>14</v>
       </c>
-      <c r="C58" s="116" t="s">
+      <c r="C58" s="84" t="s">
         <v>148</v>
       </c>
-      <c r="D58" s="84"/>
-      <c r="E58" s="84"/>
+      <c r="D58" s="103"/>
+      <c r="E58" s="103"/>
       <c r="F58" s="54"/>
       <c r="H58" s="52"/>
     </row>
     <row r="59" spans="2:8" s="34" customFormat="1" ht="15.6">
-      <c r="B59" s="115">
+      <c r="B59" s="83">
         <v>15</v>
       </c>
-      <c r="C59" s="116" t="s">
+      <c r="C59" s="84" t="s">
         <v>149</v>
       </c>
-      <c r="D59" s="84"/>
-      <c r="E59" s="84"/>
+      <c r="D59" s="103"/>
+      <c r="E59" s="103"/>
       <c r="F59" s="54"/>
       <c r="H59" s="52"/>
     </row>
     <row r="60" spans="2:8" s="34" customFormat="1" ht="15.6">
-      <c r="B60" s="115">
+      <c r="B60" s="83">
         <v>16</v>
       </c>
-      <c r="C60" s="116" t="s">
+      <c r="C60" s="84" t="s">
         <v>150</v>
       </c>
-      <c r="D60" s="84"/>
-      <c r="E60" s="84"/>
+      <c r="D60" s="103"/>
+      <c r="E60" s="103"/>
       <c r="F60" s="54"/>
       <c r="H60" s="52"/>
     </row>
     <row r="61" spans="2:8" s="34" customFormat="1" ht="15.6">
-      <c r="B61" s="115">
+      <c r="B61" s="83">
         <v>17</v>
       </c>
-      <c r="C61" s="116" t="s">
+      <c r="C61" s="84" t="s">
         <v>151</v>
       </c>
-      <c r="D61" s="84"/>
-      <c r="E61" s="84"/>
+      <c r="D61" s="103"/>
+      <c r="E61" s="103"/>
       <c r="F61" s="54"/>
       <c r="H61" s="52"/>
     </row>
     <row r="62" spans="2:8" s="34" customFormat="1" ht="15.6">
-      <c r="B62" s="115">
+      <c r="B62" s="83">
         <v>18</v>
       </c>
-      <c r="C62" s="116" t="s">
+      <c r="C62" s="84" t="s">
         <v>152</v>
       </c>
-      <c r="D62" s="84"/>
-      <c r="E62" s="84"/>
+      <c r="D62" s="103"/>
+      <c r="E62" s="103"/>
       <c r="F62" s="54"/>
       <c r="H62" s="52"/>
     </row>
     <row r="63" spans="2:8" s="34" customFormat="1" ht="15.6">
-      <c r="B63" s="115">
+      <c r="B63" s="83">
         <v>19</v>
       </c>
-      <c r="C63" s="116" t="s">
+      <c r="C63" s="84" t="s">
         <v>153</v>
       </c>
-      <c r="D63" s="84"/>
-      <c r="E63" s="84"/>
+      <c r="D63" s="103"/>
+      <c r="E63" s="103"/>
       <c r="F63" s="54"/>
       <c r="H63" s="52"/>
     </row>
     <row r="64" spans="2:8" s="34" customFormat="1" ht="15.6">
-      <c r="B64" s="115">
+      <c r="B64" s="83">
         <v>20</v>
       </c>
-      <c r="C64" s="116" t="s">
+      <c r="C64" s="84" t="s">
         <v>154</v>
       </c>
-      <c r="D64" s="84"/>
-      <c r="E64" s="84"/>
+      <c r="D64" s="103"/>
+      <c r="E64" s="103"/>
       <c r="F64" s="54"/>
       <c r="H64" s="52"/>
     </row>
     <row r="65" spans="1:8" s="34" customFormat="1" ht="15.6">
-      <c r="B65" s="115">
+      <c r="B65" s="83">
         <v>21</v>
       </c>
-      <c r="C65" s="116" t="s">
+      <c r="C65" s="84" t="s">
         <v>155</v>
       </c>
-      <c r="D65" s="84"/>
-      <c r="E65" s="84"/>
+      <c r="D65" s="103"/>
+      <c r="E65" s="103"/>
       <c r="F65" s="54"/>
       <c r="H65" s="52"/>
     </row>
     <row r="66" spans="1:8" s="34" customFormat="1" ht="15.6">
-      <c r="B66" s="115">
+      <c r="B66" s="83">
         <v>22</v>
       </c>
-      <c r="C66" s="116" t="s">
+      <c r="C66" s="84" t="s">
         <v>156</v>
       </c>
-      <c r="D66" s="84"/>
-      <c r="E66" s="84"/>
+      <c r="D66" s="103"/>
+      <c r="E66" s="103"/>
       <c r="F66" s="54"/>
       <c r="H66" s="52"/>
     </row>
     <row r="67" spans="1:8" s="34" customFormat="1" ht="15.6">
-      <c r="B67" s="115">
+      <c r="B67" s="83">
         <v>23</v>
       </c>
-      <c r="C67" s="116" t="s">
+      <c r="C67" s="84" t="s">
         <v>157</v>
       </c>
-      <c r="D67" s="84"/>
-      <c r="E67" s="84"/>
+      <c r="D67" s="103"/>
+      <c r="E67" s="103"/>
       <c r="F67" s="54"/>
       <c r="H67" s="52"/>
     </row>
     <row r="68" spans="1:8" s="34" customFormat="1" ht="15.6">
-      <c r="B68" s="115">
+      <c r="B68" s="83">
         <v>24</v>
       </c>
-      <c r="C68" s="116" t="s">
+      <c r="C68" s="84" t="s">
         <v>158</v>
       </c>
-      <c r="D68" s="84"/>
-      <c r="E68" s="84"/>
+      <c r="D68" s="103"/>
+      <c r="E68" s="103"/>
       <c r="F68" s="54"/>
       <c r="H68" s="52"/>
     </row>
     <row r="69" spans="1:8" s="34" customFormat="1" ht="15.6">
-      <c r="B69" s="115">
+      <c r="B69" s="83">
         <v>25</v>
       </c>
-      <c r="C69" s="116" t="s">
+      <c r="C69" s="84" t="s">
         <v>159</v>
       </c>
-      <c r="D69" s="84"/>
-      <c r="E69" s="84"/>
+      <c r="D69" s="103"/>
+      <c r="E69" s="103"/>
       <c r="F69" s="54"/>
       <c r="H69" s="52"/>
     </row>
     <row r="70" spans="1:8" s="34" customFormat="1" ht="15.6">
-      <c r="B70" s="115">
+      <c r="B70" s="83">
         <v>26</v>
       </c>
-      <c r="C70" s="116" t="s">
+      <c r="C70" s="84" t="s">
         <v>160</v>
       </c>
-      <c r="D70" s="84"/>
-      <c r="E70" s="84"/>
+      <c r="D70" s="103"/>
+      <c r="E70" s="103"/>
       <c r="F70" s="54"/>
       <c r="H70" s="52"/>
     </row>
     <row r="71" spans="1:8" s="34" customFormat="1" ht="15.6">
-      <c r="B71" s="115">
+      <c r="B71" s="83">
         <v>27</v>
       </c>
-      <c r="C71" s="116" t="s">
+      <c r="C71" s="84" t="s">
         <v>161</v>
       </c>
-      <c r="D71" s="84"/>
-      <c r="E71" s="84"/>
+      <c r="D71" s="103"/>
+      <c r="E71" s="103"/>
       <c r="F71" s="54"/>
       <c r="H71" s="52"/>
     </row>
     <row r="72" spans="1:8" s="34" customFormat="1" ht="15.6">
-      <c r="B72" s="115">
+      <c r="B72" s="83">
         <v>28</v>
       </c>
-      <c r="C72" s="116" t="s">
+      <c r="C72" s="84" t="s">
         <v>162</v>
       </c>
-      <c r="D72" s="84"/>
-      <c r="E72" s="84"/>
+      <c r="D72" s="103"/>
+      <c r="E72" s="103"/>
       <c r="F72" s="54"/>
       <c r="H72" s="52"/>
     </row>
     <row r="73" spans="1:8" s="34" customFormat="1" ht="15.6">
-      <c r="B73" s="111"/>
-      <c r="C73" s="112"/>
-      <c r="D73" s="113"/>
-      <c r="E73" s="113"/>
-      <c r="F73" s="114"/>
+      <c r="B73" s="58"/>
+      <c r="C73" s="59"/>
+      <c r="D73" s="60"/>
+      <c r="E73" s="60"/>
+      <c r="F73" s="61"/>
       <c r="H73" s="52"/>
     </row>
     <row r="74" spans="1:8" s="64" customFormat="1" ht="27" customHeight="1">
@@ -15197,10 +15185,10 @@
       <c r="C75" s="68" t="s">
         <v>23</v>
       </c>
-      <c r="D75" s="94" t="s">
+      <c r="D75" s="111" t="s">
         <v>24</v>
       </c>
-      <c r="E75" s="94"/>
+      <c r="E75" s="111"/>
       <c r="F75" s="68" t="s">
         <v>54</v>
       </c>
@@ -15215,10 +15203,10 @@
       <c r="C76" s="71" t="s">
         <v>80</v>
       </c>
-      <c r="D76" s="93" t="s">
+      <c r="D76" s="112" t="s">
         <v>81</v>
       </c>
-      <c r="E76" s="93"/>
+      <c r="E76" s="112"/>
       <c r="F76" s="71" t="s">
         <v>61</v>
       </c>
@@ -15233,10 +15221,10 @@
       <c r="C77" s="71" t="s">
         <v>82</v>
       </c>
-      <c r="D77" s="93" t="s">
+      <c r="D77" s="112" t="s">
         <v>83</v>
       </c>
-      <c r="E77" s="93"/>
+      <c r="E77" s="112"/>
       <c r="F77" s="71" t="s">
         <v>62</v>
       </c>
@@ -15251,10 +15239,10 @@
       <c r="C78" s="71" t="s">
         <v>84</v>
       </c>
-      <c r="D78" s="93" t="s">
+      <c r="D78" s="112" t="s">
         <v>85</v>
       </c>
-      <c r="E78" s="93"/>
+      <c r="E78" s="112"/>
       <c r="F78" s="71" t="s">
         <v>63</v>
       </c>
@@ -15269,10 +15257,10 @@
       <c r="C79" s="71" t="s">
         <v>86</v>
       </c>
-      <c r="D79" s="93" t="s">
+      <c r="D79" s="112" t="s">
         <v>87</v>
       </c>
-      <c r="E79" s="93"/>
+      <c r="E79" s="112"/>
       <c r="F79" s="71" t="s">
         <v>63</v>
       </c>
@@ -15286,10 +15274,10 @@
       <c r="C80" s="71" t="s">
         <v>88</v>
       </c>
-      <c r="D80" s="93" t="s">
+      <c r="D80" s="112" t="s">
         <v>89</v>
       </c>
-      <c r="E80" s="93"/>
+      <c r="E80" s="112"/>
       <c r="F80" s="71" t="s">
         <v>90</v>
       </c>
@@ -15303,10 +15291,10 @@
       <c r="C81" s="71" t="s">
         <v>91</v>
       </c>
-      <c r="D81" s="93" t="s">
+      <c r="D81" s="112" t="s">
         <v>92</v>
       </c>
-      <c r="E81" s="93"/>
+      <c r="E81" s="112"/>
       <c r="F81" s="71"/>
       <c r="G81" s="69"/>
     </row>
@@ -15338,10 +15326,10 @@
       <c r="C84" s="68" t="s">
         <v>23</v>
       </c>
-      <c r="D84" s="94" t="s">
+      <c r="D84" s="111" t="s">
         <v>24</v>
       </c>
-      <c r="E84" s="94"/>
+      <c r="E84" s="111"/>
       <c r="F84" s="68" t="s">
         <v>54</v>
       </c>
@@ -15361,10 +15349,10 @@
       <c r="C85" s="71" t="s">
         <v>95</v>
       </c>
-      <c r="D85" s="93" t="s">
+      <c r="D85" s="112" t="s">
         <v>96</v>
       </c>
-      <c r="E85" s="93"/>
+      <c r="E85" s="112"/>
       <c r="F85" s="71" t="s">
         <v>61</v>
       </c>
@@ -15384,10 +15372,10 @@
       <c r="C86" s="71" t="s">
         <v>97</v>
       </c>
-      <c r="D86" s="93" t="s">
+      <c r="D86" s="112" t="s">
         <v>98</v>
       </c>
-      <c r="E86" s="93"/>
+      <c r="E86" s="112"/>
       <c r="F86" s="71" t="s">
         <v>63</v>
       </c>
@@ -15401,10 +15389,10 @@
       <c r="C87" s="71" t="s">
         <v>99</v>
       </c>
-      <c r="D87" s="93" t="s">
+      <c r="D87" s="112" t="s">
         <v>100</v>
       </c>
-      <c r="E87" s="93"/>
+      <c r="E87" s="112"/>
       <c r="F87" s="71" t="s">
         <v>63</v>
       </c>
@@ -15418,10 +15406,10 @@
       <c r="C88" s="71" t="s">
         <v>101</v>
       </c>
-      <c r="D88" s="93" t="s">
+      <c r="D88" s="112" t="s">
         <v>102</v>
       </c>
-      <c r="E88" s="93"/>
+      <c r="E88" s="112"/>
       <c r="F88" s="71" t="s">
         <v>62</v>
       </c>
@@ -15435,10 +15423,10 @@
       <c r="C89" s="71" t="s">
         <v>103</v>
       </c>
-      <c r="D89" s="93" t="s">
+      <c r="D89" s="112" t="s">
         <v>104</v>
       </c>
-      <c r="E89" s="93"/>
+      <c r="E89" s="112"/>
       <c r="F89" s="71" t="s">
         <v>105</v>
       </c>
@@ -15452,10 +15440,10 @@
       <c r="C90" s="71" t="s">
         <v>91</v>
       </c>
-      <c r="D90" s="93" t="s">
+      <c r="D90" s="112" t="s">
         <v>106</v>
       </c>
-      <c r="E90" s="93"/>
+      <c r="E90" s="112"/>
       <c r="F90" s="71"/>
       <c r="G90" s="69"/>
       <c r="H90" s="62"/>
@@ -15713,41 +15701,17 @@
     </row>
   </sheetData>
   <mergeCells count="60">
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="D71:E71"/>
-    <mergeCell ref="D72:E72"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="D68:E68"/>
-    <mergeCell ref="B1:C3"/>
-    <mergeCell ref="D1:F3"/>
-    <mergeCell ref="B7:C8"/>
-    <mergeCell ref="E7:G7"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D90:E90"/>
+    <mergeCell ref="D85:E85"/>
+    <mergeCell ref="D86:E86"/>
+    <mergeCell ref="D87:E87"/>
+    <mergeCell ref="D88:E88"/>
+    <mergeCell ref="D89:E89"/>
+    <mergeCell ref="D78:E78"/>
+    <mergeCell ref="D79:E79"/>
+    <mergeCell ref="D80:E80"/>
+    <mergeCell ref="D81:E81"/>
+    <mergeCell ref="D84:E84"/>
     <mergeCell ref="D75:E75"/>
     <mergeCell ref="D76:E76"/>
     <mergeCell ref="D77:E77"/>
@@ -15762,17 +15726,41 @@
     <mergeCell ref="D61:E61"/>
     <mergeCell ref="D62:E62"/>
     <mergeCell ref="D63:E63"/>
-    <mergeCell ref="D78:E78"/>
-    <mergeCell ref="D79:E79"/>
-    <mergeCell ref="D80:E80"/>
-    <mergeCell ref="D81:E81"/>
-    <mergeCell ref="D84:E84"/>
-    <mergeCell ref="D90:E90"/>
-    <mergeCell ref="D85:E85"/>
-    <mergeCell ref="D86:E86"/>
-    <mergeCell ref="D87:E87"/>
-    <mergeCell ref="D88:E88"/>
-    <mergeCell ref="D89:E89"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="B1:C3"/>
+    <mergeCell ref="D1:F3"/>
+    <mergeCell ref="B7:C8"/>
+    <mergeCell ref="E7:G7"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="D72:E72"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="D68:E68"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F42" xr:uid="{00000000-0002-0000-0200-000000000000}">

</xml_diff>